<commit_message>
gex + skip intowall
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$12</f>
+              <f>'Daily'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$12</f>
+              <f>'Daily'!$B$2:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$12</f>
+              <f>'Daily'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$12</f>
+              <f>'Daily'!$C$2:$C$13</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-02 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-09-10 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$19)</f>
+        <f>SUM(Trades!$N$2:$N$20)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$19,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$20,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$19,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$20,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$19,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$19,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$20,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$20,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$19,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$19,"&gt;0")/SUMIF(Trades!$N$2:$N$19,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$20,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$20,"&gt;0")/SUMIF(Trades!$N$2:$N$20,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$12)</f>
+        <f>MAX(Daily!$B$2:$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$12)</f>
+        <f>MIN(Daily!$B$2:$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$19)</f>
+        <f>SUM(Trades!$R$2:$R$20)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2408,6 +2408,68 @@
         <v>3.26</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>09-10 09:53</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>09-10 10:26</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="J20" s="10" t="n"/>
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="6" t="n">
+        <v>0.1286</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>-0.6286</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>-880</v>
+      </c>
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q20" s="10" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2419,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2469,7 +2531,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -2477,11 +2539,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -2496,7 +2558,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -2504,11 +2566,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -2523,7 +2585,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -2531,11 +2593,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -2550,7 +2612,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -2558,11 +2620,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -2577,7 +2639,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -2585,11 +2647,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -2604,7 +2666,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -2612,11 +2674,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -2631,7 +2693,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -2639,11 +2701,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -2658,7 +2720,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -2666,11 +2728,11 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
@@ -2685,7 +2747,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-28")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-28")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -2693,11 +2755,11 @@
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-28")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-28")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-08-28")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-28")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F10">
@@ -2712,7 +2774,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-09-01")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-01")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -2720,11 +2782,11 @@
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-09-01")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-01")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-09-01")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-01")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F11">
@@ -2739,7 +2801,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-09-02")*Trades!$N$2:$N$19)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-02")*Trades!$N$2:$N$20)</f>
         <v/>
       </c>
       <c r="C12" s="11">
@@ -2747,15 +2809,42 @@
         <v/>
       </c>
       <c r="D12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-09-02")*(Trades!$P$2:$P$19="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-02")*(Trades!$P$2:$P$20="Closed")*1)</f>
         <v/>
       </c>
       <c r="E12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$19,"yyyy-mm-dd")="2026-09-02")*(Trades!$N$2:$N$19&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-02")*(Trades!$N$2:$N$20&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F12">
         <f>D12-E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>09/10</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-10")*Trades!$N$2:$N$20)</f>
+        <v/>
+      </c>
+      <c r="C13" s="11">
+        <f>SUM($B$2:B13)</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-10")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-10")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>D13-E13</f>
         <v/>
       </c>
     </row>
@@ -2815,15 +2904,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$B$2:$B$19,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$B$2:$B$20,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$19,A3,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$20,A3,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$19,A3,Trades!$N$2:$N$19,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$20,A3,Trades!$N$2:$N$20,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -2863,11 +2952,11 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$O$2:$O$19,A8)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIF(Trades!$O$2:$O$19,A8)</f>
+        <f>COUNTIF(Trades!$O$2:$O$20,A8)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -2882,11 +2971,11 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$O$2:$O$19,A9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIF(Trades!$O$2:$O$19,A9)</f>
+        <f>COUNTIF(Trades!$O$2:$O$20,A9)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -2901,11 +2990,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$O$2:$O$19,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$19,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$20,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -2920,11 +3009,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$O$2:$O$19,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$19,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$20,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -2963,11 +3052,11 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,9)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Trades!$G$2:$G$19,9,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,9,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2978,11 +3067,11 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,10)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Trades!$G$2:$G$19,10,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,10,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2993,11 +3082,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,11)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$19,11,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,11,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3008,11 +3097,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,12)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$19,12,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,12,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3023,11 +3112,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,13)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$19,13,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,13,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3038,11 +3127,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,14)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$19,14,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,14,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3053,11 +3142,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$G$2:$G$19,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,15)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$19,15,Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$20,15,Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3097,15 +3186,15 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$Q$2:$Q$19,A27&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$Q$2:$Q$20,A27&amp;" *")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Trades!$Q$2:$Q$19,A27&amp;" *",Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$20,A27&amp;" *",Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
       <c r="D27" s="13">
-        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$19,A27&amp;" *",Trades!$N$2:$N$19,"&gt;0")/C27)</f>
+        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$20,A27&amp;" *",Trades!$N$2:$N$20,"&gt;0")/C27)</f>
         <v/>
       </c>
     </row>
@@ -3116,15 +3205,15 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$Q$2:$Q$19,A28&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$Q$2:$Q$20,A28&amp;" *")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Trades!$Q$2:$Q$19,A28&amp;" *",Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$20,A28&amp;" *",Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
       <c r="D28" s="13">
-        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$19,A28&amp;" *",Trades!$N$2:$N$19,"&gt;0")/C28)</f>
+        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$20,A28&amp;" *",Trades!$N$2:$N$20,"&gt;0")/C28)</f>
         <v/>
       </c>
     </row>
@@ -3135,15 +3224,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$19,Trades!$Q$2:$Q$19,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$Q$2:$Q$20,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$19,A29&amp;" *",Trades!$P$2:$P$19,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$20,A29&amp;" *",Trades!$P$2:$P$20,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$19,A29&amp;" *",Trades!$N$2:$N$19,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$20,A29&amp;" *",Trades!$N$2:$N$20,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
gex and go live status
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$13</f>
+              <f>'Daily'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$13</f>
+              <f>'Daily'!$B$2:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$13</f>
+              <f>'Daily'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$13</f>
+              <f>'Daily'!$C$2:$C$14</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-10 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-09-16 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$20)</f>
+        <f>SUM(Trades!$N$2:$N$21)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$20,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$21,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$20,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$21,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$20,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$20,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$21,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$21,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$20,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$20,"&gt;0")/SUMIF(Trades!$N$2:$N$20,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$21,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$21,"&gt;0")/SUMIF(Trades!$N$2:$N$21,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$13)</f>
+        <f>MAX(Daily!$B$2:$B$14)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$13)</f>
+        <f>MIN(Daily!$B$2:$B$14)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$20)</f>
+        <f>SUM(Trades!$R$2:$R$21)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2470,6 +2470,68 @@
         <v>3.26</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>09-16 09:51</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>09-16 12:06</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>135</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="J21" s="10" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="6" t="n">
+        <v>0.3788</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>0.1515</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P21" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q21" s="10" t="inlineStr"/>
+      <c r="R21" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2481,7 +2543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2531,7 +2593,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -2539,11 +2601,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -2558,7 +2620,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -2566,11 +2628,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -2585,7 +2647,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -2593,11 +2655,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -2612,7 +2674,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -2620,11 +2682,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -2639,7 +2701,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -2647,11 +2709,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -2666,7 +2728,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -2674,11 +2736,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -2693,7 +2755,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -2701,11 +2763,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -2720,7 +2782,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -2728,11 +2790,11 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
@@ -2747,7 +2809,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-28")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-28")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -2755,11 +2817,11 @@
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-28")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-28")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-08-28")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-08-28")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F10">
@@ -2774,7 +2836,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-01")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-01")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -2782,11 +2844,11 @@
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-01")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-01")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-01")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-01")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F11">
@@ -2801,7 +2863,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-02")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-02")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C12" s="11">
@@ -2809,11 +2871,11 @@
         <v/>
       </c>
       <c r="D12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-02")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-02")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-02")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-02")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F12">
@@ -2828,7 +2890,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-10")*Trades!$N$2:$N$20)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-10")*Trades!$N$2:$N$21)</f>
         <v/>
       </c>
       <c r="C13" s="11">
@@ -2836,15 +2898,42 @@
         <v/>
       </c>
       <c r="D13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-10")*(Trades!$P$2:$P$20="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-10")*(Trades!$P$2:$P$21="Closed")*1)</f>
         <v/>
       </c>
       <c r="E13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$20,"yyyy-mm-dd")="2026-09-10")*(Trades!$N$2:$N$20&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-10")*(Trades!$N$2:$N$21&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F13">
         <f>D13-E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>09/16</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-16")*Trades!$N$2:$N$21)</f>
+        <v/>
+      </c>
+      <c r="C14" s="11">
+        <f>SUM($B$2:B14)</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-16")*(Trades!$P$2:$P$21="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$21,"yyyy-mm-dd")="2026-09-16")*(Trades!$N$2:$N$21&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>D14-E14</f>
         <v/>
       </c>
     </row>
@@ -2904,15 +2993,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$B$2:$B$20,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$B$2:$B$21,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$20,A3,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$21,A3,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$20,A3,Trades!$N$2:$N$20,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$21,A3,Trades!$N$2:$N$21,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -2952,11 +3041,11 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A8)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$O$2:$O$21,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIF(Trades!$O$2:$O$20,A8)</f>
+        <f>COUNTIF(Trades!$O$2:$O$21,A8)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -2971,11 +3060,11 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$O$2:$O$21,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIF(Trades!$O$2:$O$20,A9)</f>
+        <f>COUNTIF(Trades!$O$2:$O$21,A9)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -2990,11 +3079,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$O$2:$O$21,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$20,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$21,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -3009,11 +3098,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$O$2:$O$20,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$O$2:$O$21,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$20,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$21,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -3052,11 +3141,11 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,9)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Trades!$G$2:$G$20,9,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,9,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3067,11 +3156,11 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,10)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Trades!$G$2:$G$20,10,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,10,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3082,11 +3171,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,11)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$20,11,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,11,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3097,11 +3186,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,12)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$20,12,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,12,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3112,11 +3201,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,13)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$20,13,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,13,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3127,11 +3216,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,14)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$20,14,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,14,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3142,11 +3231,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$G$2:$G$20,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$G$2:$G$21,15)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$20,15,Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$21,15,Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3186,15 +3275,15 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$Q$2:$Q$20,A27&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$Q$2:$Q$21,A27&amp;" *")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Trades!$Q$2:$Q$20,A27&amp;" *",Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$21,A27&amp;" *",Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
       <c r="D27" s="13">
-        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$20,A27&amp;" *",Trades!$N$2:$N$20,"&gt;0")/C27)</f>
+        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$21,A27&amp;" *",Trades!$N$2:$N$21,"&gt;0")/C27)</f>
         <v/>
       </c>
     </row>
@@ -3205,15 +3294,15 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$Q$2:$Q$20,A28&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$Q$2:$Q$21,A28&amp;" *")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Trades!$Q$2:$Q$20,A28&amp;" *",Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$21,A28&amp;" *",Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
       <c r="D28" s="13">
-        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$20,A28&amp;" *",Trades!$N$2:$N$20,"&gt;0")/C28)</f>
+        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$21,A28&amp;" *",Trades!$N$2:$N$21,"&gt;0")/C28)</f>
         <v/>
       </c>
     </row>
@@ -3224,15 +3313,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$20,Trades!$Q$2:$Q$20,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$21,Trades!$Q$2:$Q$21,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$20,A29&amp;" *",Trades!$P$2:$P$20,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$21,A29&amp;" *",Trades!$P$2:$P$21,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$20,A29&amp;" *",Trades!$N$2:$N$20,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$21,A29&amp;" *",Trades!$N$2:$N$21,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
gex + trend off
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$15</f>
+              <f>'Daily'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$15</f>
+              <f>'Daily'!$B$2:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$15</f>
+              <f>'Daily'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$15</f>
+              <f>'Daily'!$C$2:$C$16</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-18 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-09-24 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$22)</f>
+        <f>SUM(Trades!$N$2:$N$24)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$22,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$24,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$22,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$24,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$22,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$22,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$24,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$24,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$22,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$22,"&gt;0")/SUMIF(Trades!$N$2:$N$22,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$24,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$24,"&gt;0")/SUMIF(Trades!$N$2:$N$24,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$15)</f>
+        <f>MAX(Daily!$B$2:$B$16)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$15)</f>
+        <f>MIN(Daily!$B$2:$B$16)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$22)</f>
+        <f>SUM(Trades!$R$2:$R$24)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2594,6 +2594,130 @@
         <v>3.26</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>09-24 09:54</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>09-24 10:10</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="J23" s="10" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="6" t="n">
+        <v>0.5455</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>0.3485</v>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>460</v>
+      </c>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P23" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q23" s="10" t="inlineStr"/>
+      <c r="R23" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>09-24 14:00</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>09-24 14:03</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" s="10" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J24" s="10" t="n"/>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>-0.4625</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>-370</v>
+      </c>
+      <c r="O24" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P24" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q24" s="10" t="inlineStr"/>
+      <c r="R24" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2605,7 +2729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2655,7 +2779,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -2663,11 +2787,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -2682,7 +2806,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -2690,11 +2814,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -2709,7 +2833,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -2717,11 +2841,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -2736,7 +2860,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -2744,11 +2868,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -2763,7 +2887,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -2771,11 +2895,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -2790,7 +2914,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -2798,11 +2922,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -2817,7 +2941,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -2825,11 +2949,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -2844,7 +2968,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -2852,11 +2976,11 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
@@ -2871,7 +2995,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-28")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-28")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -2879,11 +3003,11 @@
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-28")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-28")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-08-28")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-08-28")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F10">
@@ -2898,7 +3022,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-01")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-01")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -2906,11 +3030,11 @@
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-01")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-01")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-01")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-01")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F11">
@@ -2925,7 +3049,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-02")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-02")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C12" s="11">
@@ -2933,11 +3057,11 @@
         <v/>
       </c>
       <c r="D12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-02")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-02")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-02")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-02")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F12">
@@ -2952,7 +3076,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-10")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-10")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C13" s="11">
@@ -2960,11 +3084,11 @@
         <v/>
       </c>
       <c r="D13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-10")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-10")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-10")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-10")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F13">
@@ -2979,7 +3103,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-16")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-16")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C14" s="11">
@@ -2987,11 +3111,11 @@
         <v/>
       </c>
       <c r="D14">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-16")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-16")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E14">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-16")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-16")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F14">
@@ -3006,7 +3130,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-18")*Trades!$N$2:$N$22)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-18")*Trades!$N$2:$N$24)</f>
         <v/>
       </c>
       <c r="C15" s="11">
@@ -3014,15 +3138,42 @@
         <v/>
       </c>
       <c r="D15">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-18")*(Trades!$P$2:$P$22="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-18")*(Trades!$P$2:$P$24="Closed")*1)</f>
         <v/>
       </c>
       <c r="E15">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$22,"yyyy-mm-dd")="2026-09-18")*(Trades!$N$2:$N$22&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-18")*(Trades!$N$2:$N$24&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F15">
         <f>D15-E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09/24</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-24")*Trades!$N$2:$N$24)</f>
+        <v/>
+      </c>
+      <c r="C16" s="11">
+        <f>SUM($B$2:B16)</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-24")*(Trades!$P$2:$P$24="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$24,"yyyy-mm-dd")="2026-09-24")*(Trades!$N$2:$N$24&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>D16-E16</f>
         <v/>
       </c>
     </row>
@@ -3082,15 +3233,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$B$2:$B$22,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$B$2:$B$24,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$22,A3,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$24,A3,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$22,A3,Trades!$N$2:$N$22,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$24,A3,Trades!$N$2:$N$24,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -3130,11 +3281,11 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$O$2:$O$22,A8)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$O$2:$O$24,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIF(Trades!$O$2:$O$22,A8)</f>
+        <f>COUNTIF(Trades!$O$2:$O$24,A8)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -3149,11 +3300,11 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$O$2:$O$22,A9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$O$2:$O$24,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIF(Trades!$O$2:$O$22,A9)</f>
+        <f>COUNTIF(Trades!$O$2:$O$24,A9)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -3168,11 +3319,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$O$2:$O$22,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$O$2:$O$24,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$22,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$24,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -3187,11 +3338,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$O$2:$O$22,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$O$2:$O$24,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$22,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$24,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -3230,11 +3381,11 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,9)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Trades!$G$2:$G$22,9,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,9,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3245,11 +3396,11 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,10)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Trades!$G$2:$G$22,10,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,10,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3260,11 +3411,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,11)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$22,11,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,11,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3275,11 +3426,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,12)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$22,12,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,12,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3290,11 +3441,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,13)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$22,13,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,13,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3305,11 +3456,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,14)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$22,14,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,14,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3320,11 +3471,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$G$2:$G$22,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$G$2:$G$24,15)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$22,15,Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$24,15,Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3364,15 +3515,15 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$Q$2:$Q$22,A27&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$Q$2:$Q$24,A27&amp;" *")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Trades!$Q$2:$Q$22,A27&amp;" *",Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$24,A27&amp;" *",Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
       <c r="D27" s="13">
-        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$22,A27&amp;" *",Trades!$N$2:$N$22,"&gt;0")/C27)</f>
+        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$24,A27&amp;" *",Trades!$N$2:$N$24,"&gt;0")/C27)</f>
         <v/>
       </c>
     </row>
@@ -3383,15 +3534,15 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$Q$2:$Q$22,A28&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$Q$2:$Q$24,A28&amp;" *")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Trades!$Q$2:$Q$22,A28&amp;" *",Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$24,A28&amp;" *",Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
       <c r="D28" s="13">
-        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$22,A28&amp;" *",Trades!$N$2:$N$22,"&gt;0")/C28)</f>
+        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$24,A28&amp;" *",Trades!$N$2:$N$24,"&gt;0")/C28)</f>
         <v/>
       </c>
     </row>
@@ -3402,15 +3553,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$22,Trades!$Q$2:$Q$22,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$24,Trades!$Q$2:$Q$24,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$22,A29&amp;" *",Trades!$P$2:$P$22,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$24,A29&amp;" *",Trades!$P$2:$P$24,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$22,A29&amp;" *",Trades!$N$2:$N$22,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$24,A29&amp;" *",Trades!$N$2:$N$24,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>

</xml_diff>